<commit_message>
Refactor checks and quality scoring; add ETL modules and debug schemas
</commit_message>
<xml_diff>
--- a/testing/run/testing_files/u1_score_tests.xlsx
+++ b/testing/run/testing_files/u1_score_tests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dergun\Documents\hfqa_tool\testing\run\testing_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8360BC4A-86DF-4E86-AE90-05ACF8FFCE48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F716B70-9452-42B6-99CB-DAF76C7EDB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11835" yWindow="2730" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9675" yWindow="2385" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="U1_score_tests" sheetId="1" r:id="rId1"/>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="32">
   <si>
     <t>Site_A</t>
   </si>
   <si>
-    <t>[yes]</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -42,9 +39,6 @@
     <t>Site_B</t>
   </si>
   <si>
-    <t>[no]</t>
-  </si>
-  <si>
     <t>U4</t>
   </si>
   <si>
@@ -60,9 +54,6 @@
     <t>_results</t>
   </si>
   <si>
-    <t>C9</t>
-  </si>
-  <si>
     <t>C2</t>
   </si>
   <si>
@@ -81,29 +72,62 @@
     <t>child_u3</t>
   </si>
   <si>
-    <t>parent_inherits_worst</t>
-  </si>
-  <si>
-    <t>parent_ignores_self_uses_child</t>
-  </si>
-  <si>
     <t>k_child_1</t>
   </si>
   <si>
     <t>k_child_6</t>
   </si>
   <si>
-    <t>parent_inherits_U4</t>
-  </si>
-  <si>
-    <t>parent_no_children</t>
+    <t>_numeric_result</t>
+  </si>
+  <si>
+    <t>expected_result</t>
+  </si>
+  <si>
+    <t>over_limit_case</t>
+  </si>
+  <si>
+    <t>valid_low</t>
+  </si>
+  <si>
+    <t>Site_Z</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>child_u2</t>
+  </si>
+  <si>
+    <t>Site_X</t>
+  </si>
+  <si>
+    <t>foo</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>value_is_string</t>
+  </si>
+  <si>
+    <t>bar</t>
+  </si>
+  <si>
+    <t>uncertainty_is_string</t>
+  </si>
+  <si>
+    <t>Site_Y</t>
+  </si>
+  <si>
+    <t>missing_uncertainty</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -112,6 +136,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -136,8 +167,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -356,199 +393,289 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="36.5703125" customWidth="1"/>
+    <col min="5" max="5" width="44.140625" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" customWidth="1"/>
+    <col min="7" max="7" width="44.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>100</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
+        <v>100</v>
+      </c>
+      <c r="C3" s="1">
+        <v>20</v>
+      </c>
+      <c r="D3" s="1">
+        <v>20</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>100</v>
+      </c>
+      <c r="C4" s="1">
+        <v>30</v>
+      </c>
+      <c r="D4" s="1">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1">
+        <v>100</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1">
+        <v>4</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1">
+        <v>100</v>
+      </c>
+      <c r="C6" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="D6" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1">
+        <v>100</v>
+      </c>
+      <c r="C7" s="1">
+        <v>25.1</v>
+      </c>
+      <c r="D7" s="1">
+        <v>25.1</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1">
+        <v>100</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1">
+        <v>100</v>
+      </c>
+      <c r="C9" s="1">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>100</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3">
-        <v>100</v>
-      </c>
-      <c r="C3">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="D9" s="1">
+        <v>10</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="1">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>100</v>
-      </c>
-      <c r="C5">
+      <c r="F10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="1">
+        <v>100</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
+      <c r="B12" s="1">
+        <v>100</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E5" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6">
-        <v>100</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>2</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>100</v>
-      </c>
-      <c r="C7">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>2</v>
-      </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>100</v>
-      </c>
-      <c r="C8">
-        <v>25.1</v>
-      </c>
-      <c r="D8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>6</v>
-      </c>
-      <c r="F8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="F12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10">
-        <v>100</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+      <c r="G12" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>